<commit_message>
Increasing iled of wind offshore, adding back hydro
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr updateLinks="never"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\SubRES_Tmpl\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C48DD9-DED7-479B-A74E-1DB16C47A208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43D1AB6C-6213-44E6-95F9-17D6D986C9C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28702" yWindow="-98" windowWidth="28995" windowHeight="15675" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVA" sheetId="6" r:id="rId1"/>
@@ -591,14 +591,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{268E9BAB-B98F-4B82-9042-51EABC9ED525}">
   <dimension ref="B3:C5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>21</v>
       </c>
@@ -606,7 +606,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>59</v>
       </c>
@@ -622,24 +622,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3954DD3-0F24-46DF-B268-7A98442D0282}">
   <dimension ref="A1:O13"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.59765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.59765625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.19921875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.46484375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.9296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.86328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="4.73046875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.90625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="4.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -686,7 +686,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -733,7 +733,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>44</v>
       </c>
@@ -780,7 +780,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>44</v>
       </c>
@@ -827,7 +827,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -874,7 +874,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -921,7 +921,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -968,7 +968,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -1015,7 +1015,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>44</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>44</v>
       </c>
@@ -1109,7 +1109,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -1156,7 +1156,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -1203,7 +1203,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>44</v>
       </c>
@@ -1258,21 +1258,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="C4:X50"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="13.3984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7265625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.86328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.3984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.73046875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.7265625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.26953125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="4" spans="3:24" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>4</v>
       </c>
@@ -1286,7 +1287,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="5" spans="3:24" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>3</v>
       </c>
@@ -1312,7 +1313,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="6" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D6" t="s">
         <v>6</v>
       </c>
@@ -1332,7 +1333,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="7" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D7" t="s">
         <v>7</v>
       </c>
@@ -1352,7 +1353,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="8" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D8" t="s">
         <v>8</v>
       </c>
@@ -1363,7 +1364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="9" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D9" t="s">
         <v>9</v>
       </c>
@@ -1374,7 +1375,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="10" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="10" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D10" t="s">
         <v>10</v>
       </c>
@@ -1385,7 +1386,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="11" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D11" t="s">
         <v>6</v>
       </c>
@@ -1399,7 +1400,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="12" spans="3:24" x14ac:dyDescent="0.35">
       <c r="P12" s="2" t="s">
         <v>25</v>
       </c>
@@ -1416,7 +1417,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="13" spans="3:24" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
         <v>4</v>
       </c>
@@ -1443,7 +1444,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="14" spans="3:24" x14ac:dyDescent="0.35">
       <c r="C14" t="s">
         <v>3</v>
       </c>
@@ -1482,7 +1483,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="15" spans="3:24" x14ac:dyDescent="0.35">
       <c r="C15" t="s">
         <v>11</v>
       </c>
@@ -1521,7 +1522,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="16" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D16" t="s">
         <v>6</v>
       </c>
@@ -1554,7 +1555,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="17" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D17" t="s">
         <v>13</v>
       </c>
@@ -1562,7 +1563,7 @@
         <v>55</v>
       </c>
       <c r="G17">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>30</v>
@@ -1589,7 +1590,7 @@
         <v>EN[_]Hydro*</v>
       </c>
     </row>
-    <row r="18" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="18" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D18" t="s">
         <v>13</v>
       </c>
@@ -1624,7 +1625,7 @@
         <v>E[_]SPV*</v>
       </c>
     </row>
-    <row r="19" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="19" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D19" t="s">
         <v>7</v>
       </c>
@@ -1659,7 +1660,7 @@
         <v>E[_]WOF*</v>
       </c>
     </row>
-    <row r="20" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="20" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D20" t="s">
         <v>8</v>
       </c>
@@ -1694,7 +1695,7 @@
         <v>E[_]WON*</v>
       </c>
     </row>
-    <row r="21" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="21" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D21" t="s">
         <v>9</v>
       </c>
@@ -1729,7 +1730,7 @@
         <v>EN[_]Hydro*</v>
       </c>
     </row>
-    <row r="22" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="22" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D22" t="s">
         <v>10</v>
       </c>
@@ -1764,18 +1765,18 @@
         <v>E[_]SPV*</v>
       </c>
     </row>
-    <row r="23" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="23" spans="3:24" x14ac:dyDescent="0.35">
       <c r="P23" s="2" t="s">
         <v>31</v>
       </c>
       <c r="Q23" s="2">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="R23" s="2">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="S23" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T23" t="str">
         <f t="shared" si="2"/>
@@ -1790,7 +1791,7 @@
         <v>E[_]WOF*</v>
       </c>
     </row>
-    <row r="24" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="24" spans="3:24" x14ac:dyDescent="0.35">
       <c r="P24" s="2" t="s">
         <v>31</v>
       </c>
@@ -1816,12 +1817,12 @@
         <v>E[_]WON*</v>
       </c>
     </row>
-    <row r="27" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="27" spans="3:24" x14ac:dyDescent="0.35">
       <c r="C27" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="28" spans="3:24" x14ac:dyDescent="0.35">
       <c r="C28" t="s">
         <v>16</v>
       </c>
@@ -1838,7 +1839,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="29" spans="3:24" x14ac:dyDescent="0.35">
       <c r="C29" t="s">
         <v>17</v>
       </c>
@@ -1849,7 +1850,7 @@
         <v>8.76</v>
       </c>
     </row>
-    <row r="30" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="30" spans="3:24" x14ac:dyDescent="0.35">
       <c r="C30" t="s">
         <v>53</v>
       </c>
@@ -1860,7 +1861,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="31" spans="3:24" x14ac:dyDescent="0.35">
       <c r="C31" t="s">
         <v>17</v>
       </c>
@@ -1871,7 +1872,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="32" spans="3:24" x14ac:dyDescent="0.45">
+    <row r="32" spans="3:24" x14ac:dyDescent="0.35">
       <c r="D32" t="s">
         <v>7</v>
       </c>
@@ -1882,7 +1883,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="33" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="33" spans="3:7" x14ac:dyDescent="0.35">
       <c r="D33" t="s">
         <v>10</v>
       </c>
@@ -1893,7 +1894,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="3:7" x14ac:dyDescent="0.35">
       <c r="D34" t="s">
         <v>9</v>
       </c>
@@ -1904,7 +1905,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C35" t="s">
         <v>17</v>
       </c>
@@ -1918,12 +1919,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C38" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C39" t="s">
         <v>21</v>
       </c>
@@ -1934,7 +1935,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="40" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="40" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C40" t="s">
         <v>14</v>
       </c>
@@ -1945,7 +1946,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="41" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C41" t="s">
         <v>15</v>
       </c>
@@ -1956,7 +1957,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="42" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C42" t="s">
         <v>57</v>
       </c>
@@ -1967,7 +1968,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="43" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C43" t="s">
         <v>55</v>
       </c>
@@ -1978,7 +1979,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="44" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C44" t="s">
         <v>56</v>
       </c>
@@ -1989,12 +1990,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="47" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="47" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C47" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="3:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C48" t="s">
         <v>1</v>
       </c>
@@ -2008,7 +2009,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="49" spans="3:6" x14ac:dyDescent="0.45">
+    <row r="49" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C49" t="s">
         <v>64</v>
       </c>
@@ -2022,7 +2023,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="50" spans="3:6" x14ac:dyDescent="0.45">
+    <row r="50" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C50" t="s">
         <v>69</v>
       </c>

</xml_diff>

<commit_message>
Correcting start - aggregated plants are still allowed to invest in 2025
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122E2282-E13A-4C8F-81F2-984ED8B29792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA66A3B0-EA48-4807-AEE4-0137691D7686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="77">
   <si>
     <t>PSET_PN</t>
   </si>
@@ -244,6 +244,9 @@
     <t>-pasti</t>
   </si>
   <si>
+    <t>solar,wind,coal,gas,nuclear,hydro,bioenergy</t>
+  </si>
+  <si>
     <t>life</t>
   </si>
   <si>
@@ -262,7 +265,10 @@
     <t>ELC_wo*</t>
   </si>
   <si>
-    <t>solar,wind,coal,gas,nuclear,hydro,bioenergy,ElcAgg_Solar,ElcAgg_Wind</t>
+    <t>pset_pn</t>
+  </si>
+  <si>
+    <t>ElcAgg_Solar,ElcAgg_Wind</t>
   </si>
 </sst>
 </file>
@@ -1257,7 +1263,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="C4:X50"/>
+  <dimension ref="C4:X55"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -1951,7 +1957,7 @@
         <v>15</v>
       </c>
       <c r="D41" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E41" t="s">
         <v>24</v>
@@ -1973,7 +1979,7 @@
         <v>55</v>
       </c>
       <c r="D43" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E43" t="s">
         <v>24</v>
@@ -1984,7 +1990,7 @@
         <v>56</v>
       </c>
       <c r="D44" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E44" t="s">
         <v>24</v>
@@ -2020,21 +2026,54 @@
         <v>67</v>
       </c>
       <c r="F49" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="50" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C50" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D50">
         <v>40</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F50" t="s">
-        <v>70</v>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="53" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C53" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C54" t="s">
+        <v>1</v>
+      </c>
+      <c r="D54" t="s">
+        <v>26</v>
+      </c>
+      <c r="E54" t="s">
+        <v>66</v>
+      </c>
+      <c r="F54" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="55" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C55" t="s">
+        <v>64</v>
+      </c>
+      <c r="D55">
+        <v>2030</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F55" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Battery investments allowed from 2030
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA66A3B0-EA48-4807-AEE4-0137691D7686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32057E53-71D9-411C-B03A-C35A805DC39B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -268,7 +268,7 @@
     <t>pset_pn</t>
   </si>
   <si>
-    <t>ElcAgg_Solar,ElcAgg_Wind</t>
+    <t>ElcAgg_Solar,ElcAgg_Wind,EN_STG8hbNREL,EN_STG4hbNREL</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Updating cap_bnd of won and sol
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C5DFB5-017C-463C-B32E-A0131E436DE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5347D07B-8601-4082-A133-E856B33DFCC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1831,13 +1831,13 @@
         <v>77</v>
       </c>
       <c r="Q25" s="2">
-        <v>1400</v>
+        <v>1.4</v>
       </c>
       <c r="R25" s="2">
-        <v>1400</v>
+        <v>1.4</v>
       </c>
       <c r="S25" s="2">
-        <v>1400</v>
+        <v>1.4</v>
       </c>
       <c r="T25" t="s">
         <v>56</v>
@@ -1848,13 +1848,13 @@
         <v>77</v>
       </c>
       <c r="Q26" s="2">
-        <v>1500</v>
+        <v>1.5</v>
       </c>
       <c r="R26" s="2">
-        <v>1500</v>
+        <v>1.5</v>
       </c>
       <c r="S26" s="2">
-        <v>1500</v>
+        <v>1.5</v>
       </c>
       <c r="T26" t="str">
         <f t="shared" si="2"/>

</xml_diff>

<commit_message>
oil shale ban failed because who can come up with a model where a simple capacity retirement as scenario can be so difficult - trying to add capacity restriction to wind and pv instead meanwhile
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5347D07B-8601-4082-A133-E856B33DFCC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E67F262-9C8C-414C-9AD5-3C3A01D7E25E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="78">
   <si>
     <t>PSET_PN</t>
   </si>
@@ -271,7 +271,7 @@
     <t>ElcAgg_Solar,ElcAgg_Wind,EN_STG8hbNREL,EN_STG4hbNREL</t>
   </si>
   <si>
-    <t>cap_bnd~up</t>
+    <t>EST</t>
   </si>
 </sst>
 </file>
@@ -1280,6 +1280,7 @@
     <col min="13" max="13" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="4.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="3:24" x14ac:dyDescent="0.25">
@@ -1622,7 +1623,7 @@
         <v>16</v>
       </c>
       <c r="T18" t="str">
-        <f t="shared" ref="T18:T26" si="2">T14</f>
+        <f t="shared" ref="T18:T24" si="2">T14</f>
         <v>E[_]SPV*</v>
       </c>
       <c r="W18" t="str">
@@ -1826,45 +1827,24 @@
         <v>E[_]WON*</v>
       </c>
     </row>
-    <row r="25" spans="3:24" x14ac:dyDescent="0.25">
-      <c r="P25" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="Q25" s="2">
-        <v>1.4</v>
-      </c>
-      <c r="R25" s="2">
-        <v>1.4</v>
-      </c>
-      <c r="S25" s="2">
-        <v>1.4</v>
-      </c>
-      <c r="T25" t="s">
-        <v>56</v>
-      </c>
-    </row>
     <row r="26" spans="3:24" x14ac:dyDescent="0.25">
       <c r="P26" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="Q26" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="R26" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="S26" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="T26" t="str">
-        <f t="shared" si="2"/>
-        <v>E[_]SPV*</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="3:24" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
         <v>4</v>
       </c>
+      <c r="P27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>0</v>
+      </c>
+      <c r="R27" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="28" spans="3:24" x14ac:dyDescent="0.25">
       <c r="C28" t="s">
@@ -1882,6 +1862,15 @@
       <c r="G28" t="s">
         <v>5</v>
       </c>
+      <c r="P28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>56</v>
+      </c>
+      <c r="R28">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="29" spans="3:24" x14ac:dyDescent="0.25">
       <c r="C29" t="s">
@@ -1892,6 +1881,15 @@
       </c>
       <c r="G29" s="1">
         <v>8.76</v>
+      </c>
+      <c r="P29" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>57</v>
+      </c>
+      <c r="R29">
+        <v>1.5</v>
       </c>
     </row>
     <row r="30" spans="3:24" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Aggregate removed from start = 2030
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr updateLinks="never"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B8A52E-0258-453E-B017-838171EC8405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59920AF4-B74E-4B32-9652-DAD1DC895DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="78">
   <si>
     <t>PSET_PN</t>
   </si>
@@ -268,7 +268,10 @@
     <t>pset_pn</t>
   </si>
   <si>
-    <t>ElcAgg_Solar,ElcAgg_Wind,EN_STG8hbNREL,EN_STG4hbNREL</t>
+    <t>EN_STG8hbNREL,EN_STG4hbNREL</t>
+  </si>
+  <si>
+    <t>ElcAgg_Solar,ElcAgg_Wind,</t>
   </si>
 </sst>
 </file>
@@ -2022,7 +2025,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="49" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C49" t="s">
         <v>64</v>
       </c>
@@ -2036,7 +2039,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="50" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C50" t="s">
         <v>69</v>
       </c>
@@ -2050,12 +2053,12 @@
         <v>71</v>
       </c>
     </row>
-    <row r="53" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C53" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C54" t="s">
         <v>1</v>
       </c>
@@ -2069,7 +2072,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="55" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C55" t="s">
         <v>64</v>
       </c>
@@ -2081,6 +2084,9 @@
       </c>
       <c r="F55" t="s">
         <v>76</v>
+      </c>
+      <c r="H55" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Connecting Estonia's demand to harku
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59920AF4-B74E-4B32-9652-DAD1DC895DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94ABFF6F-C524-4630-99BF-1DC563923188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVA" sheetId="6" r:id="rId1"/>
@@ -37,8 +37,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={1BF36063-6E02-40C0-ACF0-91FBA8E0608D}</author>
+  </authors>
+  <commentList>
+    <comment ref="C45" authorId="0" shapeId="0" xr:uid="{1BF36063-6E02-40C0-ACF0-91FBA8E0608D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Single demand process connected to harku for now</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="82">
   <si>
     <t>PSET_PN</t>
   </si>
@@ -272,13 +290,25 @@
   </si>
   <si>
     <t>ElcAgg_Solar,ElcAgg_Wind,</t>
+  </si>
+  <si>
+    <t>e_demand</t>
+  </si>
+  <si>
+    <t>~tfm_topins</t>
+  </si>
+  <si>
+    <t>e_harku_330</t>
+  </si>
+  <si>
+    <t>e_demand_agg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -292,6 +322,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -334,6 +370,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Kristopher Raik" id="{1A26B760-FB54-48F1-8363-71FD6F653EC5}" userId="S::krraik@taltech.ee::b956339b-354b-46f9-8dd3-3584d8dbf762" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -597,17 +639,31 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="C45" dT="2026-03-17T14:42:24.14" personId="{1A26B760-FB54-48F1-8363-71FD6F653EC5}" id="{1BF36063-6E02-40C0-ACF0-91FBA8E0608D}">
+    <text>Single demand process connected to harku for now</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{268E9BAB-B98F-4B82-9042-51EABC9ED525}">
-  <dimension ref="B3:C5"/>
+  <dimension ref="B3:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>21</v>
       </c>
@@ -615,12 +671,39 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>59</v>
       </c>
       <c r="C5">
         <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D16" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1265,12 +1348,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="C4:X55"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="41.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -2006,6 +2089,17 @@
         <v>24</v>
       </c>
     </row>
+    <row r="45" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C45" t="s">
+        <v>78</v>
+      </c>
+      <c r="D45" t="s">
+        <v>80</v>
+      </c>
+      <c r="E45" t="s">
+        <v>24</v>
+      </c>
+    </row>
     <row r="47" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C47" t="s">
         <v>4</v>
@@ -2092,6 +2186,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Correct start time of fermi nuclear
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A79143AB-3EFE-413A-A153-48F6C6FB4B51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED7709A2-1A65-4FE6-8EF2-D59611DB93BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="82">
   <si>
     <t>PSET_PN</t>
   </si>
@@ -317,6 +317,9 @@
   </si>
   <si>
     <t>FERMI NUCLEAR</t>
+  </si>
+  <si>
+    <t>~TFM_UPD</t>
   </si>
 </sst>
 </file>
@@ -2132,21 +2135,13 @@
         <v>55</v>
       </c>
     </row>
-    <row r="36" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="P36" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q36">
-        <v>2036</v>
-      </c>
-      <c r="R36" t="s">
-        <v>80</v>
-      </c>
-    </row>
     <row r="38" spans="3:18" x14ac:dyDescent="0.25">
       <c r="C38" t="s">
         <v>20</v>
       </c>
+      <c r="P38" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="39" spans="3:18" x14ac:dyDescent="0.25">
       <c r="C39" t="s">
@@ -2157,6 +2152,15 @@
       </c>
       <c r="E39" t="s">
         <v>23</v>
+      </c>
+      <c r="P39" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q39">
+        <v>2036</v>
+      </c>
+      <c r="R39" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="40" spans="3:18" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Moved comment rows out from  Pset_PN under "Attribute" column
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr updateLinks="never"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A43350-D461-41B5-8F5E-D185526C1F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D992C96-FDE9-4B7A-B27A-C618BD6D1AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="40" windowWidth="19200" windowHeight="11240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVA" sheetId="6" r:id="rId1"/>
@@ -447,7 +447,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="14">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{9640D755-0D23-4E24-A066-51A16F3F8D30}"/>
@@ -762,20 +762,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{268E9BAB-B98F-4B82-9042-51EABC9ED525}">
   <dimension ref="B3:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="49.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>19</v>
       </c>
@@ -783,7 +783,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>35</v>
       </c>
@@ -799,28 +799,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:V70"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7265625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="31.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.26953125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.7265625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="28.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="31.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
@@ -839,7 +839,7 @@
       <c r="O2" s="5"/>
       <c r="P2" s="5"/>
     </row>
-    <row r="3" spans="2:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="8" t="s">
         <v>54</v>
       </c>
@@ -886,12 +886,12 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="J4" s="11" t="s">
+    <row r="4" spans="2:22" x14ac:dyDescent="0.35">
+      <c r="D4" s="11" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:22" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>10</v>
       </c>
@@ -908,7 +908,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D6" t="s">
         <v>5</v>
       </c>
@@ -919,7 +919,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D7" t="s">
         <v>12</v>
       </c>
@@ -930,7 +930,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D8" t="s">
         <v>12</v>
       </c>
@@ -941,7 +941,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D9" t="s">
         <v>6</v>
       </c>
@@ -952,7 +952,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D10" t="s">
         <v>7</v>
       </c>
@@ -963,7 +963,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D11" t="s">
         <v>8</v>
       </c>
@@ -974,7 +974,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D12" t="s">
         <v>9</v>
       </c>
@@ -989,12 +989,12 @@
       <c r="T12" s="2"/>
       <c r="V12" s="2"/>
     </row>
-    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="J13" s="11" t="s">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.35">
+      <c r="D13" s="11" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D14" t="s">
         <v>5</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D15" t="s">
         <v>6</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D16" t="s">
         <v>7</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:18" x14ac:dyDescent="0.35">
       <c r="D17" t="s">
         <v>8</v>
       </c>
@@ -1038,7 +1038,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:18" x14ac:dyDescent="0.35">
       <c r="D18" t="s">
         <v>9</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:18" x14ac:dyDescent="0.35">
       <c r="D19" t="s">
         <v>5</v>
       </c>
@@ -1060,12 +1060,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="J20" s="11" t="s">
+    <row r="20" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="D20" s="11" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="21" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:18" x14ac:dyDescent="0.35">
       <c r="D21" t="s">
         <v>5</v>
       </c>
@@ -1076,7 +1076,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:18" x14ac:dyDescent="0.35">
       <c r="D22" t="s">
         <v>7</v>
       </c>
@@ -1087,7 +1087,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:18" x14ac:dyDescent="0.35">
       <c r="D23" t="s">
         <v>16</v>
       </c>
@@ -1098,7 +1098,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:18" x14ac:dyDescent="0.35">
       <c r="D24" t="s">
         <v>6</v>
       </c>
@@ -1109,7 +1109,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:18" x14ac:dyDescent="0.35">
       <c r="D25" t="s">
         <v>9</v>
       </c>
@@ -1120,7 +1120,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:18" x14ac:dyDescent="0.35">
       <c r="D26" t="s">
         <v>8</v>
       </c>
@@ -1131,7 +1131,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:18" x14ac:dyDescent="0.35">
       <c r="D27" t="s">
         <v>11</v>
       </c>
@@ -1145,13 +1145,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:18" x14ac:dyDescent="0.35">
       <c r="R28" s="2"/>
     </row>
-    <row r="29" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:18" x14ac:dyDescent="0.35">
       <c r="R29" s="2"/>
     </row>
-    <row r="32" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B32" s="7" t="s">
         <v>3</v>
       </c>
@@ -1159,7 +1159,7 @@
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
     </row>
-    <row r="33" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B33" s="8" t="s">
         <v>54</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D34" t="s">
         <v>40</v>
       </c>
@@ -1196,7 +1196,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D35" t="s">
         <v>40</v>
       </c>
@@ -1207,7 +1207,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D36" t="s">
         <v>40</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="37" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D37" t="s">
         <v>40</v>
       </c>
@@ -1229,7 +1229,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="38" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D38" t="s">
         <v>40</v>
       </c>
@@ -1243,7 +1243,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D39" t="s">
         <v>42</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D40" t="s">
         <v>40</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B46" s="7" t="s">
         <v>28</v>
       </c>
@@ -1279,7 +1279,7 @@
       <c r="D46" s="4"/>
       <c r="E46" s="4"/>
     </row>
-    <row r="47" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B47" s="8" t="s">
         <v>54</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="48" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D48" s="2" t="s">
         <v>21</v>
       </c>
@@ -1332,7 +1332,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="49" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D49" s="2" t="s">
         <v>21</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D50" s="2" t="s">
         <v>21</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D51" s="2" t="s">
         <v>21</v>
       </c>
@@ -1413,7 +1413,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D52" s="2" t="s">
         <v>22</v>
       </c>
@@ -1442,7 +1442,7 @@
         <v>EN[_]Hydro*</v>
       </c>
     </row>
-    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D53" s="2" t="s">
         <v>22</v>
       </c>
@@ -1471,7 +1471,7 @@
         <v>E[_]SPV*</v>
       </c>
     </row>
-    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D54" s="2" t="s">
         <v>22</v>
       </c>
@@ -1500,7 +1500,7 @@
         <v>E[_]WOF*</v>
       </c>
     </row>
-    <row r="55" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D55" s="2" t="s">
         <v>22</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>E[_]WON*</v>
       </c>
     </row>
-    <row r="56" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D56" s="2" t="s">
         <v>23</v>
       </c>
@@ -1558,7 +1558,7 @@
         <v>EN[_]Hydro*</v>
       </c>
     </row>
-    <row r="57" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D57" s="2" t="s">
         <v>23</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>E[_]SPV*</v>
       </c>
     </row>
-    <row r="58" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D58" s="2" t="s">
         <v>23</v>
       </c>
@@ -1616,7 +1616,7 @@
         <v>E[_]WOF*</v>
       </c>
     </row>
-    <row r="59" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D59" s="2" t="s">
         <v>23</v>
       </c>
@@ -1645,7 +1645,7 @@
         <v>E[_]WON*</v>
       </c>
     </row>
-    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D60" s="2" t="s">
         <v>48</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="61" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D61" s="2" t="s">
         <v>48</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D62" s="2" t="s">
         <v>48</v>
       </c>
@@ -1705,7 +1705,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="64" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B64" s="7" t="s">
         <v>18</v>
       </c>
@@ -1713,7 +1713,7 @@
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
     </row>
-    <row r="65" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B65" s="12" t="s">
         <v>69</v>
       </c>
@@ -1727,7 +1727,7 @@
       <c r="F65" s="14"/>
       <c r="J65" s="13"/>
     </row>
-    <row r="66" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
         <v>13</v>
       </c>
@@ -1738,7 +1738,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="67" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
         <v>14</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="68" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
         <v>33</v>
       </c>
@@ -1760,7 +1760,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="69" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
         <v>31</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="70" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
         <v>32</v>
       </c>

</xml_diff>

<commit_message>
Removed EN_STG 4H and 8H conditions from SubRES_New_RE_and_Conventional_Trans.xlsx file because this is a deprecated element
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_EST/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D992C96-FDE9-4B7A-B27A-C618BD6D1AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B24621C-47C9-4BB7-9FBD-A9B12784A57F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="40" windowWidth="19200" windowHeight="11240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
     <author>tc={9326A9B6-D94C-4ED3-9FB8-434C0D4AC388}</author>
   </authors>
   <commentList>
-    <comment ref="I49" authorId="0" shapeId="0" xr:uid="{80A2C193-6148-4AA7-9B62-06322F60E0BF}">
+    <comment ref="I48" authorId="0" shapeId="0" xr:uid="{80A2C193-6148-4AA7-9B62-06322F60E0BF}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -52,7 +52,7 @@
     Utility-scale PV</t>
       </text>
     </comment>
-    <comment ref="I50" authorId="1" shapeId="0" xr:uid="{E6F93F18-BBEF-4E19-B2D0-A493D668847A}">
+    <comment ref="I49" authorId="1" shapeId="0" xr:uid="{E6F93F18-BBEF-4E19-B2D0-A493D668847A}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -60,7 +60,7 @@
     AC fixed</t>
       </text>
     </comment>
-    <comment ref="I61" authorId="2" shapeId="0" xr:uid="{9326A9B6-D94C-4ED3-9FB8-434C0D4AC388}">
+    <comment ref="I60" authorId="2" shapeId="0" xr:uid="{9326A9B6-D94C-4ED3-9FB8-434C0D4AC388}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="72">
   <si>
     <t>Attribute</t>
   </si>
@@ -214,9 +214,6 @@
   </si>
   <si>
     <t>ELC_wo*</t>
-  </si>
-  <si>
-    <t>EN_STG8hbNREL,EN_STG4hbNREL</t>
   </si>
   <si>
     <t>act_cost</t>
@@ -747,13 +744,13 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="I49" dT="2026-03-18T13:56:27.06" personId="{50AE587C-9924-43E9-9BB9-052BDB346AE2}" id="{80A2C193-6148-4AA7-9B62-06322F60E0BF}">
+  <threadedComment ref="I48" dT="2026-03-18T13:56:27.06" personId="{50AE587C-9924-43E9-9BB9-052BDB346AE2}" id="{80A2C193-6148-4AA7-9B62-06322F60E0BF}">
     <text>Utility-scale PV</text>
   </threadedComment>
-  <threadedComment ref="I50" dT="2026-03-18T13:39:46.05" personId="{50AE587C-9924-43E9-9BB9-052BDB346AE2}" id="{E6F93F18-BBEF-4E19-B2D0-A493D668847A}">
+  <threadedComment ref="I49" dT="2026-03-18T13:39:46.05" personId="{50AE587C-9924-43E9-9BB9-052BDB346AE2}" id="{E6F93F18-BBEF-4E19-B2D0-A493D668847A}">
     <text>AC fixed</text>
   </threadedComment>
-  <threadedComment ref="I61" dT="2026-03-18T13:39:46.05" personId="{50AE587C-9924-43E9-9BB9-052BDB346AE2}" id="{9326A9B6-D94C-4ED3-9FB8-434C0D4AC388}">
+  <threadedComment ref="I60" dT="2026-03-18T13:39:46.05" personId="{50AE587C-9924-43E9-9BB9-052BDB346AE2}" id="{9326A9B6-D94C-4ED3-9FB8-434C0D4AC388}">
     <text>AC fixed</text>
   </threadedComment>
 </ThreadedComments>
@@ -798,7 +795,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:V70"/>
+  <dimension ref="B2:V69"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14.1796875" bestFit="1" customWidth="1"/>
@@ -806,7 +803,7 @@
     <col min="4" max="4" width="12.7265625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="41.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.453125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="31.1796875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
@@ -841,7 +838,7 @@
     </row>
     <row r="3" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>2</v>
@@ -856,39 +853,39 @@
         <v>4</v>
       </c>
       <c r="G3" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="I3" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="J3" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="K3" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="L3" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="M3" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="N3" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="O3" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="P3" s="9" t="s">
         <v>63</v>
-      </c>
-      <c r="P3" s="9" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="4" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D4" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="2:22" x14ac:dyDescent="0.35">
@@ -991,7 +988,7 @@
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D13" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.35">
@@ -1062,7 +1059,7 @@
     </row>
     <row r="20" spans="2:18" x14ac:dyDescent="0.35">
       <c r="D20" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="2:18" x14ac:dyDescent="0.35">
@@ -1161,7 +1158,7 @@
     </row>
     <row r="33" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B33" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>2</v>
@@ -1173,16 +1170,16 @@
         <v>1</v>
       </c>
       <c r="F33" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G33" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G33" s="12" t="s">
+      <c r="H33" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="H33" s="9" t="s">
-        <v>70</v>
-      </c>
       <c r="I33" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.35">
@@ -1193,7 +1190,7 @@
         <v>2030</v>
       </c>
       <c r="G34" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.35">
@@ -1215,7 +1212,7 @@
         <v>2036</v>
       </c>
       <c r="G36" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.35">
@@ -1226,7 +1223,7 @@
         <v>2030</v>
       </c>
       <c r="G37" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.35">
@@ -1240,7 +1237,7 @@
         <v>41</v>
       </c>
       <c r="I38" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.35">
@@ -1254,55 +1251,68 @@
         <v>43</v>
       </c>
       <c r="I39" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="D40" t="s">
-        <v>40</v>
-      </c>
-      <c r="F40">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="45" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B45" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+    </row>
+    <row r="46" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B46" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="E46" s="10">
+        <v>2023</v>
+      </c>
+      <c r="F46" s="10">
         <v>2030</v>
       </c>
-      <c r="G40" t="s">
-        <v>47</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B46" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
-    </row>
-    <row r="47" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C47" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="E47" s="10">
-        <v>2023</v>
-      </c>
-      <c r="F47" s="10">
-        <v>2030</v>
-      </c>
-      <c r="G47" s="10">
+      <c r="G46" s="10">
         <v>2040</v>
       </c>
-      <c r="H47" s="10">
+      <c r="H46" s="10">
         <v>2050</v>
       </c>
-      <c r="I47" s="12" t="s">
-        <v>69</v>
+      <c r="I46" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="47" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="D47" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E47" s="2">
+        <v>2700</v>
+      </c>
+      <c r="F47" s="2">
+        <v>2700</v>
+      </c>
+      <c r="G47" s="2">
+        <v>2700</v>
+      </c>
+      <c r="H47" s="2">
+        <v>2700</v>
+      </c>
+      <c r="I47" t="str">
+        <f>M47</f>
+        <v>EN[_]Hydro*</v>
+      </c>
+      <c r="L47" t="s">
+        <v>24</v>
+      </c>
+      <c r="M47" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.35">
@@ -1310,26 +1320,26 @@
         <v>21</v>
       </c>
       <c r="E48" s="2">
-        <v>2700</v>
+        <v>560</v>
       </c>
       <c r="F48" s="2">
-        <v>2700</v>
-      </c>
-      <c r="G48" s="2">
-        <v>2700</v>
+        <v>380</v>
+      </c>
+      <c r="G48">
+        <v>320</v>
       </c>
       <c r="H48" s="2">
-        <v>2700</v>
+        <v>290</v>
       </c>
       <c r="I48" t="str">
-        <f>M48</f>
-        <v>EN[_]Hydro*</v>
+        <f t="shared" ref="I48:I50" si="0">M48</f>
+        <v>E[_]SPV*</v>
       </c>
       <c r="L48" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M48" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.35">
@@ -1337,26 +1347,26 @@
         <v>21</v>
       </c>
       <c r="E49" s="2">
-        <v>560</v>
+        <v>2780</v>
       </c>
       <c r="F49" s="2">
-        <v>380</v>
-      </c>
-      <c r="G49">
-        <v>320</v>
+        <v>2390</v>
+      </c>
+      <c r="G49" s="2">
+        <v>2140</v>
       </c>
       <c r="H49" s="2">
-        <v>290</v>
+        <v>1990</v>
       </c>
       <c r="I49" t="str">
-        <f t="shared" ref="I49:I51" si="0">M49</f>
-        <v>E[_]SPV*</v>
+        <f t="shared" si="0"/>
+        <v>E[_]WOF*</v>
       </c>
       <c r="L49" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M49" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="50" spans="2:13" x14ac:dyDescent="0.35">
@@ -1364,53 +1374,55 @@
         <v>21</v>
       </c>
       <c r="E50" s="2">
-        <v>2780</v>
+        <v>1180</v>
       </c>
       <c r="F50" s="2">
-        <v>2390</v>
+        <v>1150</v>
       </c>
       <c r="G50" s="2">
-        <v>2140</v>
+        <v>1110</v>
       </c>
       <c r="H50" s="2">
-        <v>1990</v>
+        <v>1090</v>
       </c>
       <c r="I50" t="str">
         <f t="shared" si="0"/>
-        <v>E[_]WOF*</v>
+        <v>E[_]WON*</v>
       </c>
       <c r="L50" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M50" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="51" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D51" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E51" s="2">
-        <v>1180</v>
+        <v>70</v>
       </c>
       <c r="F51" s="2">
-        <v>1150</v>
+        <v>65</v>
       </c>
       <c r="G51" s="2">
-        <v>1110</v>
+        <v>65</v>
       </c>
       <c r="H51" s="2">
-        <v>1090</v>
+        <v>65</v>
       </c>
       <c r="I51" t="str">
-        <f t="shared" si="0"/>
-        <v>E[_]WON*</v>
-      </c>
-      <c r="L51" t="s">
-        <v>27</v>
-      </c>
-      <c r="M51" t="s">
-        <v>32</v>
+        <f>I47</f>
+        <v>EN[_]Hydro*</v>
+      </c>
+      <c r="L51" t="str">
+        <f>L47</f>
+        <v>Hydropower - large-scale unit</v>
+      </c>
+      <c r="M51" t="str">
+        <f t="shared" ref="M51:M58" si="1">M47</f>
+        <v>EN[_]Hydro*</v>
       </c>
     </row>
     <row r="52" spans="2:13" x14ac:dyDescent="0.35">
@@ -1418,28 +1430,28 @@
         <v>22</v>
       </c>
       <c r="E52" s="2">
-        <v>70</v>
+        <v>11.5</v>
       </c>
       <c r="F52" s="2">
-        <v>65</v>
+        <v>9.5</v>
       </c>
       <c r="G52" s="2">
-        <v>65</v>
+        <v>8.1</v>
       </c>
       <c r="H52" s="2">
-        <v>65</v>
+        <v>7.4</v>
       </c>
       <c r="I52" t="str">
-        <f>I48</f>
-        <v>EN[_]Hydro*</v>
+        <f t="shared" ref="I52:I58" si="2">I48</f>
+        <v>E[_]SPV*</v>
       </c>
       <c r="L52" t="str">
-        <f>L48</f>
-        <v>Hydropower - large-scale unit</v>
+        <f t="shared" ref="L52" si="3">L48</f>
+        <v>Solar photovoltaics - Large scale unit</v>
       </c>
       <c r="M52" t="str">
-        <f t="shared" ref="M52:M59" si="1">M48</f>
-        <v>EN[_]Hydro*</v>
+        <f t="shared" si="1"/>
+        <v>E[_]SPV*</v>
       </c>
     </row>
     <row r="53" spans="2:13" x14ac:dyDescent="0.35">
@@ -1447,28 +1459,28 @@
         <v>22</v>
       </c>
       <c r="E53" s="2">
-        <v>11.5</v>
+        <v>44</v>
       </c>
       <c r="F53" s="2">
-        <v>9.5</v>
+        <v>34</v>
       </c>
       <c r="G53" s="2">
-        <v>8.1</v>
+        <v>30</v>
       </c>
       <c r="H53" s="2">
-        <v>7.4</v>
+        <v>28</v>
       </c>
       <c r="I53" t="str">
-        <f t="shared" ref="I53:I59" si="2">I49</f>
-        <v>E[_]SPV*</v>
+        <f t="shared" si="2"/>
+        <v>E[_]WOF*</v>
       </c>
       <c r="L53" t="str">
-        <f t="shared" ref="L53" si="3">L49</f>
-        <v>Solar photovoltaics - Large scale unit</v>
+        <f t="shared" ref="L53" si="4">L49</f>
+        <v>Wind offshore</v>
       </c>
       <c r="M53" t="str">
         <f t="shared" si="1"/>
-        <v>E[_]SPV*</v>
+        <v>E[_]WOF*</v>
       </c>
     </row>
     <row r="54" spans="2:13" x14ac:dyDescent="0.35">
@@ -1476,57 +1488,57 @@
         <v>22</v>
       </c>
       <c r="E54" s="2">
-        <v>44</v>
+        <v>17.387</v>
       </c>
       <c r="F54" s="2">
-        <v>34</v>
+        <v>16.663</v>
       </c>
       <c r="G54" s="2">
-        <v>30</v>
+        <v>15.965</v>
       </c>
       <c r="H54" s="2">
-        <v>28</v>
+        <v>15.602</v>
       </c>
       <c r="I54" t="str">
         <f t="shared" si="2"/>
-        <v>E[_]WOF*</v>
+        <v>E[_]WON*</v>
       </c>
       <c r="L54" t="str">
-        <f t="shared" ref="L54" si="4">L50</f>
-        <v>Wind offshore</v>
+        <f t="shared" ref="L54" si="5">L50</f>
+        <v>Wind onshore</v>
       </c>
       <c r="M54" t="str">
         <f t="shared" si="1"/>
-        <v>E[_]WOF*</v>
+        <v>E[_]WON*</v>
       </c>
     </row>
     <row r="55" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D55" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E55" s="2">
-        <v>17.387</v>
+        <v>4</v>
       </c>
       <c r="F55" s="2">
-        <v>16.663</v>
+        <v>4</v>
       </c>
       <c r="G55" s="2">
-        <v>15.965</v>
+        <v>4</v>
       </c>
       <c r="H55" s="2">
-        <v>15.602</v>
+        <v>4</v>
       </c>
       <c r="I55" t="str">
         <f t="shared" si="2"/>
-        <v>E[_]WON*</v>
+        <v>EN[_]Hydro*</v>
       </c>
       <c r="L55" t="str">
-        <f t="shared" ref="L55" si="5">L51</f>
-        <v>Wind onshore</v>
+        <f t="shared" ref="L55" si="6">L51</f>
+        <v>Hydropower - large-scale unit</v>
       </c>
       <c r="M55" t="str">
         <f t="shared" si="1"/>
-        <v>E[_]WON*</v>
+        <v>EN[_]Hydro*</v>
       </c>
     </row>
     <row r="56" spans="2:13" x14ac:dyDescent="0.35">
@@ -1534,28 +1546,28 @@
         <v>23</v>
       </c>
       <c r="E56" s="2">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="F56" s="2">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="G56" s="2">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="H56" s="2">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="I56" t="str">
         <f t="shared" si="2"/>
-        <v>EN[_]Hydro*</v>
+        <v>E[_]SPV*</v>
       </c>
       <c r="L56" t="str">
-        <f t="shared" ref="L56" si="6">L52</f>
-        <v>Hydropower - large-scale unit</v>
+        <f t="shared" ref="L56" si="7">L52</f>
+        <v>Solar photovoltaics - Large scale unit</v>
       </c>
       <c r="M56" t="str">
         <f t="shared" si="1"/>
-        <v>EN[_]Hydro*</v>
+        <v>E[_]SPV*</v>
       </c>
     </row>
     <row r="57" spans="2:13" x14ac:dyDescent="0.35">
@@ -1563,28 +1575,28 @@
         <v>23</v>
       </c>
       <c r="E57" s="2">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="F57" s="2">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
       <c r="G57" s="2">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
       <c r="H57" s="2">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
       <c r="I57" t="str">
         <f t="shared" si="2"/>
-        <v>E[_]SPV*</v>
+        <v>E[_]WOF*</v>
       </c>
       <c r="L57" t="str">
-        <f t="shared" ref="L57" si="7">L53</f>
-        <v>Solar photovoltaics - Large scale unit</v>
+        <f t="shared" ref="L57" si="8">L53</f>
+        <v>Wind offshore</v>
       </c>
       <c r="M57" t="str">
         <f t="shared" si="1"/>
-        <v>E[_]SPV*</v>
+        <v>E[_]WOF*</v>
       </c>
     </row>
     <row r="58" spans="2:13" x14ac:dyDescent="0.35">
@@ -1592,193 +1604,164 @@
         <v>23</v>
       </c>
       <c r="E58" s="2">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="F58" s="2">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="G58" s="2">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="H58" s="2">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="I58" t="str">
         <f t="shared" si="2"/>
-        <v>E[_]WOF*</v>
+        <v>E[_]WON*</v>
       </c>
       <c r="L58" t="str">
-        <f t="shared" ref="L58" si="8">L54</f>
-        <v>Wind offshore</v>
+        <f t="shared" ref="L58" si="9">L54</f>
+        <v>Wind onshore</v>
       </c>
       <c r="M58" t="str">
         <f t="shared" si="1"/>
-        <v>E[_]WOF*</v>
+        <v>E[_]WON*</v>
       </c>
     </row>
     <row r="59" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D59" s="2" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="E59" s="2">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="F59" s="2">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="G59" s="2">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H59" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="I59" t="str">
-        <f t="shared" si="2"/>
-        <v>E[_]WON*</v>
-      </c>
-      <c r="L59" t="str">
-        <f t="shared" ref="L59" si="9">L55</f>
-        <v>Wind onshore</v>
-      </c>
-      <c r="M59" t="str">
-        <f t="shared" si="1"/>
-        <v>E[_]WON*</v>
+        <v>0</v>
+      </c>
+      <c r="I59" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="60" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D60" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E60" s="2">
-        <v>0</v>
+        <v>4.41</v>
       </c>
       <c r="F60" s="2">
-        <v>0</v>
+        <v>3.45</v>
       </c>
       <c r="G60" s="2">
-        <v>0</v>
+        <v>3.16</v>
       </c>
       <c r="H60" s="2">
-        <v>0</v>
+        <v>2.99</v>
       </c>
       <c r="I60" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="61" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D61" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E61" s="2">
-        <v>4.41</v>
+        <v>2.06</v>
       </c>
       <c r="F61" s="2">
-        <v>3.45</v>
+        <v>1.98</v>
       </c>
       <c r="G61" s="2">
-        <v>3.16</v>
+        <v>1.89</v>
       </c>
       <c r="H61" s="2">
-        <v>2.99</v>
+        <v>1.85</v>
       </c>
       <c r="I61" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="62" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="D62" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E62" s="2">
-        <v>2.06</v>
-      </c>
-      <c r="F62" s="2">
-        <v>1.98</v>
-      </c>
-      <c r="G62" s="2">
-        <v>1.89</v>
-      </c>
-      <c r="H62" s="2">
-        <v>1.85</v>
-      </c>
-      <c r="I62" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="64" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B64" s="7" t="s">
+    <row r="63" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B63" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C64" s="4"/>
-      <c r="D64" s="4"/>
-      <c r="E64" s="4"/>
-    </row>
-    <row r="65" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B65" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="C65" s="12" t="s">
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+    </row>
+    <row r="64" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B64" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C64" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="D64" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="D65" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="E65" s="14"/>
-      <c r="F65" s="14"/>
-      <c r="J65" s="13"/>
-    </row>
-    <row r="66" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="E64" s="14"/>
+      <c r="F64" s="14"/>
+      <c r="J64" s="13"/>
+    </row>
+    <row r="65" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B65" t="s">
+        <v>13</v>
+      </c>
+      <c r="C65" t="s">
+        <v>37</v>
+      </c>
+      <c r="D65" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="66" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C66" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="D66" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="67" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="C67" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D67" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="68" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C68" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="D68" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="69" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C69" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D69" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="70" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B70" t="s">
-        <v>32</v>
-      </c>
-      <c r="C70" t="s">
-        <v>45</v>
-      </c>
-      <c r="D70" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>